<commit_message>
Ordinal probit reparameterization: lognormal priors, dashboard improvements, data loss fix
Stan model: replace softplus(theta) transform with direct w ~ Lognormal(log(default), 1.0)
priors on lower=0 constrained parameters. No hidden transforms — posterior draws ARE the
utility weights. w_removal > w_remove_ceo_overwhelming constraint preserved via delta_removal.

Dashboard: remove obsolete Bayesian/Anchored subtitle, rename Pr(w>0.1) to Pr(relevant)
with tooltip, add Prior column showing posterior shrinkage (data-driven vs prior-sensitive).

Fix compute_phi_matrix dropping Likert observations when scenario feasible_actions changed
after elicitation (S1_062 Drev_commission_review: 50 observations were silently discarded).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/governance_spec.xlsx
+++ b/data/governance_spec.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="node_order" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="action_sets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vote_thresholds" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="utilities_board" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="utilities_asa" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="utilities_ceo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="policy_parameters" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="board_overconfidence" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="node_order" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="action_sets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="vote_thresholds" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="utilities_board" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="utilities_asa" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="utilities_ceo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="policy_parameters" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="board_overconfidence" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1230,7 +1230,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1280,7 +1280,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>0.3439</v>
       </c>
     </row>
     <row r="9">
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>0.411</v>
       </c>
     </row>
     <row r="10">
@@ -1310,7 +1310,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.5</v>
+        <v>0.8572</v>
       </c>
     </row>
     <row r="11">
@@ -1320,7 +1320,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>0.300267</v>
       </c>
     </row>
     <row r="12">
@@ -1330,7 +1330,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>0.187667</v>
       </c>
     </row>
     <row r="13">
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>0.8951</v>
       </c>
     </row>
     <row r="15">
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>0.07506699999999999</v>
       </c>
     </row>
     <row r="16">
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>0.5709</v>
       </c>
     </row>
     <row r="17">
@@ -1380,7 +1380,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.4</v>
+        <v>0.0024</v>
       </c>
     </row>
     <row r="18">
@@ -1390,7 +1390,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.5</v>
+        <v>0.1205</v>
       </c>
     </row>
     <row r="19">
@@ -1400,7 +1400,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ASA 7-dimensional utility function and 5-path Beta strike priors
Replace ad-hoc additive ASA utility with 7-dimensional weighted assessment
(FW, PPL, TD, EGR, BA, OL, PF) from asa_bayesian_params.md. Base scores
are path-dependent (CEO resign/stay × D1 action), with post-A2 adjustments
for vote, review, CEO removal, and market alignment outcomes.

Replace 3-tier ASA strike Beta priors with 5-path priors conditioned on
the full game path: Beta(18,2), Beta(14,3), Beta(24,1), Beta(15,2),
Beta(9,6) for the five A2 nodes.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/governance_spec.xlsx
+++ b/data/governance_spec.xlsx
@@ -1424,7 +1424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1442,47 +1442,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>vote_reward_weight</t>
+          <t>strike_ba_shift</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ceo_removal_reward</t>
+          <t>strike_ol_shift</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>review_car_weight</t>
+          <t>overwhelming_ba_shift</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mobilisation_cost</t>
+          <t>overwhelming_ol_shift</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>reputational_gain_weight</t>
+          <t>ceo_removal_ba_shift</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1492,31 +1492,71 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>overwhelming_reward_weight</t>
+          <t>ceo_removal_fw_shift</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>early_ceo_departure_reward</t>
+          <t>negative_review_td_shift</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>market_alignment_bonus</t>
+          <t>negative_review_egr_shift</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>balanced_review_td_shift</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>market_alignment_ol_shift</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>market_alignment_pf_shift</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>mobilisation_cost</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>